<commit_message>
feat: semana 2 de maio.
Adição e atualização das demandas de maio e ajuste de pendencias.
</commit_message>
<xml_diff>
--- a/dados-status.xlsx
+++ b/dados-status.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Status Semanal" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Semanal'!$A$1:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Status Semanal'!$A$1:$K$12</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,9 +18,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -44,7 +43,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00102A43"/>
+        <fgColor rgb="000F766E"/>
       </patternFill>
     </fill>
   </fills>
@@ -57,6 +56,15 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="00D9E1EC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9E1EC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E1EC"/>
+      </top>
       <bottom style="thin">
         <color rgb="00D9E1EC"/>
       </bottom>
@@ -65,15 +73,21 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -441,20 +455,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="64" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="72" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="58" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Atividade</t>
@@ -495,23 +512,38 @@
           <t>Observações</t>
         </is>
       </c>
-    </row>
-    <row r="2">
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Ganho</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>% Ganho</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prorrogação de títulos de revenda FOB (e DDF)</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="C2" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D2" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="E2" s="3" t="n"/>
+          <t>Prorrogação de títulos de revenda FOB e DDF</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="n">
+        <v>46146</v>
+      </c>
+      <c r="C2" s="5" t="n">
+        <v>46150</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>46149</v>
+      </c>
+      <c r="E2" s="5" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Em andamento</t>
@@ -522,29 +554,44 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Análise de aderência, AS IS e mapeamento de falhas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
+          <t>EFP finalizada e enviada ao solicitante em 07/05/2026 para validação de aderência. Aguardando de acordo; recobrar em 11/05/2026 no primeiro horário.</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Eficiência operacional</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Padronização da prorrogação e redução de retrabalho entre solicitante e financeiro.</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="3" ht="72" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Autorização para pagamento de título (adiantamento)</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="C3" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D3" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="E3" s="3" t="n"/>
+      <c r="B3" s="5" t="n">
+        <v>46146</v>
+      </c>
+      <c r="C3" s="5" t="n">
+        <v>46149</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>46149</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>46149</v>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G3" s="2" t="n">
@@ -552,27 +599,40 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Em análise operacional.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
+          <t>Demanda inclusa na prorrogação de títulos FOB e DDF. Concluída com sucesso em 07/05/2026; autorização feita pelo financeiro após ajuste da data do título pós cobrança do fornecedor.</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Gestão e controle</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Maior controle do fluxo de autorização e da data do título pelo setor financeiro.</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="4" ht="72" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Painel Analítico - Produto importado</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="C4" s="3" t="n">
-        <v>46142</v>
-      </c>
-      <c r="D4" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="E4" s="3" t="n">
-        <v>46142</v>
+          <t>Fluxo FOB Sanni</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n">
+        <v>46146</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>46151</v>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>46146</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>46151</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -584,27 +644,40 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>MCO padrão escritório e liberado para CQ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
+          <t>Concluída. Pendente criação de card no ClickUp para notificar Talita sobre a realização do CQ.</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Eficiência operacional</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Fluxo formalizado para reduzir dúvidas operacionais e acelerar o controle de qualidade.</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="5" ht="72" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Ajuste Vídeo Separação</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>46142</v>
-      </c>
-      <c r="D5" s="3" t="n">
-        <v>46140</v>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>46142</v>
+          <t>Política de avaria - recebimento (CD e Loja)</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>46139</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>46141</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>46141</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>46141</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -616,26 +689,39 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Correções realizadas e vídeo reenviado para CQ.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
+          <t>Concluída com sucesso em 29/04/2026.</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Conformidade</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Reforço da aderência à política de avarias no recebimento do CD e das lojas.</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="6" ht="72" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Política de avaria - Recebimento (CD e Loja)</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="C6" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>46141</v>
-      </c>
-      <c r="E6" s="3" t="n"/>
+          <t>Regra regime atacadista</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>46153</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>46157</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E6" s="5" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Em andamento</t>
@@ -646,29 +732,40 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Análise de cobertura MCO vs Política e identificação de lacunas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
+          <t>MCO completo. Pendente envio da ETP pelo time de sistemas, explicando o funcionamento da regra atacadista de Fortaleza. Previsão de envio: 13/05/2026.</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Conformidade</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Aplicação correta da regra atacadista e redução de risco operacional/fiscal.</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="7" ht="72" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Fluxo FOB Sanni</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="C7" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="E7" s="3" t="n"/>
+          <t>Monitor de Entrega</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>46153</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>46157</v>
+      </c>
+      <c r="D7" s="5" t="n"/>
+      <c r="E7" s="5" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>A fazer</t>
         </is>
       </c>
       <c r="G7" s="2" t="n">
@@ -676,57 +773,89 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Confecção, envio para CQ e ajustes no MCO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
+          <t>Documentações ainda não iniciadas. Análise de aderência havia sido iniciada e pausada para foco em demandas já concluídas. Demanda reclassificada como a fazer.</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Gestão e controle</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Visibilidade do acompanhamento de entregas, gargalos e pendências operacionais.</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="8" ht="72" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Regra regime atacadista</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="n">
+          <t>App separação</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
         <v>46139</v>
       </c>
-      <c r="C8" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D8" s="3" t="n"/>
-      <c r="E8" s="3" t="n"/>
+      <c r="C8" s="5" t="n">
+        <v>46141</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>46141</v>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>A fazer</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G8" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Aguardando ETP para início do MCO.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
+          <t>Concluído.</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Eficiência operacional</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Apoio à rotina de separação e redução de esforço manual no processo.</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="9" ht="72" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Monitor de entrega</t>
-        </is>
-      </c>
-      <c r="B9" s="3" t="n">
-        <v>46141</v>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>46143</v>
-      </c>
-      <c r="D9" s="3" t="n">
-        <v>46141</v>
-      </c>
-      <c r="E9" s="3" t="n"/>
+          <t>Painel analítico - produto importado</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>46139</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>46142</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>46139</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>46142</v>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Em andamento</t>
+          <t>Finalizada</t>
         </is>
       </c>
       <c r="G9" s="2" t="n">
@@ -734,31 +863,42 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Contato com solicitante para entendimento.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
+          <t>Concluído.</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Gestão e controle</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Melhor leitura gerencial dos produtos importados e apoio à tomada de decisão.</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>0.35</v>
+      </c>
+    </row>
+    <row r="10" ht="72" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>App separação</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>46141</v>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>46139</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>46141</v>
-      </c>
+          <t>Acompanhamento da migração da plataforma Weni - Suri</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>46153</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>46157</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E10" s="5" t="n"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Finalizada</t>
+          <t>Em andamento</t>
         </is>
       </c>
       <c r="G10" s="2" t="n">
@@ -766,12 +906,113 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Demanda em produção e chamado finalizado.</t>
-        </is>
+          <t>Acompanhar a migração da plataforma Weni para Suri durante a semana 11/05 a 15/05.</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Redução de custo</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Transição acompanhada para reduzir impacto operacional e capturar ganhos da nova plataforma.</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="11" ht="72" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Confecção da jornada do financeiro da plataforma Suri</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>46153</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>46157</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>46153</v>
+      </c>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Em andamento</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Confecção da jornada do financeiro na plataforma Suri em andamento. Início planejado e real em 11/05/2026; fim real será atualizado quando a demanda for concluída.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Eficiência operacional</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Jornada desenhada para orientar o financeiro e reduzir dúvidas na operação da plataforma.</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="12" ht="72" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Ajuste Vídeo Separação</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>46142</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>46140</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>46142</v>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Finalizada</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Correções realizadas e vídeo reenviado para CQ.</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Eficiência operacional</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Material corrigido e reenviado para CQ, reduzindo retrabalho no alinhamento da operação.</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>0.15</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H10"/>
+  <autoFilter ref="A1:K12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>